<commit_message>
Added new page test cases and modified and added Element Utils and test classes
</commit_message>
<xml_diff>
--- a/test/resources/testdata/excels/MasterTestData.xlsx
+++ b/test/resources/testdata/excels/MasterTestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dileep_K\Desktop\DCP_18\FrameworkPOM-master\src\test\resources\testdata\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9054152E-3A72-4BEA-8034-386BC10E87EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC694F7-8E8D-4880-B69A-5161A02BB987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{01F410BB-4CDF-4E65-BF55-31489716C62E}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="80">
   <si>
     <t>TC101</t>
   </si>
@@ -213,9 +213,6 @@
     <t>Logged in as John Doe</t>
   </si>
   <si>
-    <t>kilhklikjop0eg8079093@ixunbo.com</t>
-  </si>
-  <si>
     <t>TC105</t>
   </si>
   <si>
@@ -262,6 +259,27 @@
   </si>
   <si>
     <t>C:\Users\Dileep_K\Desktop</t>
+  </si>
+  <si>
+    <t>Name On Card</t>
+  </si>
+  <si>
+    <t>Kanna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Card Number </t>
+  </si>
+  <si>
+    <t>CVV</t>
+  </si>
+  <si>
+    <t>Expiry Month</t>
+  </si>
+  <si>
+    <t>Expiry Year</t>
+  </si>
+  <si>
+    <t>kilhklikjop0g8070093@ixunbo.com</t>
   </si>
 </sst>
 </file>
@@ -641,7 +659,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADC914BC-115C-4E99-A655-A098063134BC}">
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:Z20"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="26" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.08984375" style="3" bestFit="1" customWidth="1"/>
@@ -663,10 +681,16 @@
     <col min="18" max="18" width="32.36328125" style="3" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="36.26953125" style="3" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="31.90625" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="16384" width="8.90625" style="3"/>
+    <col min="21" max="21" width="8.90625" style="3"/>
+    <col min="22" max="22" width="23.26953125" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="33.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="8.90625" style="3"/>
+    <col min="25" max="25" width="21.7265625" style="3" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="18" style="3" bestFit="1" customWidth="1"/>
+    <col min="27" max="16384" width="8.90625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -677,7 +701,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -688,7 +712,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
@@ -714,7 +738,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
@@ -740,7 +764,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
@@ -748,7 +772,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>18</v>
       </c>
@@ -756,7 +780,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>21</v>
       </c>
@@ -817,8 +841,23 @@
       <c r="T10" s="3" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="V10" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="W10" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="X10" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y10" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="Z10" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>21</v>
       </c>
@@ -826,7 +865,7 @@
         <v>23</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>24</v>
@@ -879,41 +918,56 @@
       <c r="T11" s="3" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="V11" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="W11" s="3">
+        <v>98712345678</v>
+      </c>
+      <c r="X11" s="3">
+        <v>98</v>
+      </c>
+      <c r="Y11" s="3">
+        <v>11</v>
+      </c>
+      <c r="Z11" s="3">
+        <v>2090</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>59</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D14" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
-        <v>63</v>
-      </c>
       <c r="B16" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>2</v>
@@ -921,53 +975,53 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="C17" s="4" t="s">
         <v>64</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>67</v>
-      </c>
       <c r="C20" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deleted few files, added RetryAnalyzer, Page classes and Test classes.
</commit_message>
<xml_diff>
--- a/test/resources/testdata/excels/MasterTestData.xlsx
+++ b/test/resources/testdata/excels/MasterTestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dileep_K\Desktop\DCP_18\FrameworkPOM-master\src\test\resources\testdata\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC694F7-8E8D-4880-B69A-5161A02BB987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A91F0EF0-C627-43FE-AE7C-09B077447578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{01F410BB-4CDF-4E65-BF55-31489716C62E}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="81">
   <si>
     <t>TC101</t>
   </si>
@@ -231,12 +231,6 @@
     <t>TC106</t>
   </si>
   <si>
-    <t>haxape@gmail.com</t>
-  </si>
-  <si>
-    <t>Welcome@1234</t>
-  </si>
-  <si>
     <t>TC107</t>
   </si>
   <si>
@@ -280,6 +274,15 @@
   </si>
   <si>
     <t>kilhklikjop0g8070093@ixunbo.com</t>
+  </si>
+  <si>
+    <t>cefir28081@daerdy.com</t>
+  </si>
+  <si>
+    <t>Logged in As</t>
+  </si>
+  <si>
+    <t>cred</t>
   </si>
 </sst>
 </file>
@@ -842,19 +845,19 @@
         <v>54</v>
       </c>
       <c r="V10" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="W10" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="W10" s="3" t="s">
+      <c r="X10" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="Y10" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="X10" s="3" t="s">
+      <c r="Z10" s="3" t="s">
         <v>76</v>
-      </c>
-      <c r="Y10" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="Z10" s="3" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.35">
@@ -865,7 +868,7 @@
         <v>23</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>24</v>
@@ -919,7 +922,7 @@
         <v>55</v>
       </c>
       <c r="V11" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="W11" s="3">
         <v>98712345678</v>
@@ -972,21 +975,27 @@
       <c r="C16" s="3" t="s">
         <v>2</v>
       </c>
+      <c r="D16" s="3" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>62</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>64</v>
+        <v>24</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>22</v>
@@ -995,33 +1004,33 @@
         <v>58</v>
       </c>
       <c r="D19" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E19" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="F19" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>59</v>
       </c>
       <c r="D20" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E20" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="F20" s="3" t="s">
         <v>70</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>